<commit_message>
tried multiples params better results
</commit_message>
<xml_diff>
--- a/results/excel_reports/mobilenet_v2_resnet50_black.xlsx
+++ b/results/excel_reports/mobilenet_v2_resnet50_black.xlsx
@@ -1242,61 +1242,61 @@
         <v>0.86</v>
       </c>
       <c r="C2" t="n">
-        <v>0.838</v>
+        <v>0.842</v>
       </c>
       <c r="D2" t="n">
-        <v>0.829</v>
+        <v>0.833</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="F2" t="n">
-        <v>0.787</v>
+        <v>0.805</v>
       </c>
       <c r="G2" t="n">
-        <v>0.771</v>
+        <v>0.786</v>
       </c>
       <c r="H2" t="n">
-        <v>0.758</v>
+        <v>0.762</v>
       </c>
       <c r="I2" t="n">
-        <v>0.727</v>
+        <v>0.749</v>
       </c>
       <c r="J2" t="n">
-        <v>0.705</v>
+        <v>0.724</v>
       </c>
       <c r="K2" t="n">
-        <v>0.667</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="L2" t="n">
-        <v>0.629</v>
+        <v>0.655</v>
       </c>
       <c r="M2" t="n">
-        <v>0.585</v>
+        <v>0.621</v>
       </c>
       <c r="N2" t="n">
-        <v>0.535</v>
+        <v>0.547</v>
       </c>
       <c r="O2" t="n">
-        <v>0.475</v>
+        <v>0.5</v>
       </c>
       <c r="P2" t="n">
-        <v>0.411</v>
+        <v>0.43</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.342</v>
+        <v>0.37</v>
       </c>
       <c r="R2" t="n">
-        <v>0.275</v>
+        <v>0.29</v>
       </c>
       <c r="S2" t="n">
-        <v>0.206</v>
+        <v>0.211</v>
       </c>
       <c r="T2" t="n">
-        <v>0.118</v>
+        <v>0.127</v>
       </c>
       <c r="U2" t="n">
-        <v>0.048</v>
+        <v>0.051</v>
       </c>
       <c r="V2" t="n">
         <v>0.001</v>

</xml_diff>

<commit_message>
refactor and run again
</commit_message>
<xml_diff>
--- a/results/excel_reports/mobilenet_v2_resnet50_black.xlsx
+++ b/results/excel_reports/mobilenet_v2_resnet50_black.xlsx
@@ -752,134 +752,6 @@
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="18"/>
-          <order val="18"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A20</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$20:$V$20</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="19"/>
-          <order val="19"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A21</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$21:$V$21</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="20"/>
-          <order val="20"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A22</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$22:$V$22</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="21"/>
-          <order val="21"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A23</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$23:$V$23</f>
-            </numRef>
-          </val>
-        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -953,7 +825,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>25</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9000000" cy="5400000"/>
@@ -1263,7 +1135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -1363,68 +1235,68 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>U2Net-Saliency</t>
+          <t>random_baseline</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>0.86</v>
       </c>
       <c r="C2" t="n">
-        <v>0.835</v>
+        <v>0.379</v>
       </c>
       <c r="D2" t="n">
-        <v>0.82</v>
+        <v>0.307</v>
       </c>
       <c r="E2" t="n">
-        <v>0.806</v>
+        <v>0.221</v>
       </c>
       <c r="F2" t="n">
-        <v>0.781</v>
+        <v>0.154</v>
       </c>
       <c r="G2" t="n">
-        <v>0.758</v>
+        <v>0.109</v>
       </c>
       <c r="H2" t="n">
-        <v>0.73</v>
+        <v>0.079</v>
       </c>
       <c r="I2" t="n">
-        <v>0.715</v>
+        <v>0.054</v>
       </c>
       <c r="J2" t="n">
-        <v>0.677</v>
+        <v>0.046</v>
       </c>
       <c r="K2" t="n">
-        <v>0.65</v>
+        <v>0.032</v>
       </c>
       <c r="L2" t="n">
-        <v>0.629</v>
+        <v>0.024</v>
       </c>
       <c r="M2" t="n">
-        <v>0.572</v>
+        <v>0.022</v>
       </c>
       <c r="N2" t="n">
-        <v>0.522</v>
+        <v>0.014</v>
       </c>
       <c r="O2" t="n">
-        <v>0.471</v>
+        <v>0.012</v>
       </c>
       <c r="P2" t="n">
-        <v>0.415</v>
+        <v>0.008</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.351</v>
+        <v>0.005</v>
       </c>
       <c r="R2" t="n">
-        <v>0.263</v>
+        <v>0.001</v>
       </c>
       <c r="S2" t="n">
-        <v>0.183</v>
+        <v>0.003</v>
       </c>
       <c r="T2" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0.039</v>
+        <v>0.001</v>
       </c>
       <c r="V2" t="n">
         <v>0.001</v>
@@ -1433,68 +1305,68 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dinov2_COMBO_ENT_SMOOTH</t>
+          <t>saliency</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>0.86</v>
       </c>
       <c r="C3" t="n">
-        <v>0.852</v>
+        <v>0.597</v>
       </c>
       <c r="D3" t="n">
-        <v>0.83</v>
+        <v>0.478</v>
       </c>
       <c r="E3" t="n">
-        <v>0.826</v>
+        <v>0.408</v>
       </c>
       <c r="F3" t="n">
-        <v>0.805</v>
+        <v>0.322</v>
       </c>
       <c r="G3" t="n">
-        <v>0.796</v>
+        <v>0.263</v>
       </c>
       <c r="H3" t="n">
-        <v>0.774</v>
+        <v>0.219</v>
       </c>
       <c r="I3" t="n">
-        <v>0.756</v>
+        <v>0.177</v>
       </c>
       <c r="J3" t="n">
-        <v>0.723</v>
+        <v>0.145</v>
       </c>
       <c r="K3" t="n">
-        <v>0.694</v>
+        <v>0.13</v>
       </c>
       <c r="L3" t="n">
-        <v>0.663</v>
+        <v>0.104</v>
       </c>
       <c r="M3" t="n">
-        <v>0.612</v>
+        <v>0.074</v>
       </c>
       <c r="N3" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.06</v>
       </c>
       <c r="O3" t="n">
-        <v>0.518</v>
+        <v>0.046</v>
       </c>
       <c r="P3" t="n">
-        <v>0.435</v>
+        <v>0.028</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.367</v>
+        <v>0.014</v>
       </c>
       <c r="R3" t="n">
-        <v>0.295</v>
+        <v>0.01</v>
       </c>
       <c r="S3" t="n">
-        <v>0.212</v>
+        <v>0.006</v>
       </c>
       <c r="T3" t="n">
-        <v>0.123</v>
+        <v>0.003</v>
       </c>
       <c r="U3" t="n">
-        <v>0.051</v>
+        <v>0</v>
       </c>
       <c r="V3" t="n">
         <v>0.001</v>
@@ -1503,68 +1375,68 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>dinov2_COMBO_FIXED</t>
+          <t>guided_backprop</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>0.86</v>
       </c>
       <c r="C4" t="n">
-        <v>0.821</v>
+        <v>0.594</v>
       </c>
       <c r="D4" t="n">
-        <v>0.801</v>
+        <v>0.479</v>
       </c>
       <c r="E4" t="n">
-        <v>0.77</v>
+        <v>0.403</v>
       </c>
       <c r="F4" t="n">
-        <v>0.763</v>
+        <v>0.327</v>
       </c>
       <c r="G4" t="n">
-        <v>0.736</v>
+        <v>0.267</v>
       </c>
       <c r="H4" t="n">
-        <v>0.71</v>
+        <v>0.216</v>
       </c>
       <c r="I4" t="n">
-        <v>0.675</v>
+        <v>0.18</v>
       </c>
       <c r="J4" t="n">
-        <v>0.626</v>
+        <v>0.15</v>
       </c>
       <c r="K4" t="n">
-        <v>0.588</v>
+        <v>0.13</v>
       </c>
       <c r="L4" t="n">
-        <v>0.536</v>
+        <v>0.104</v>
       </c>
       <c r="M4" t="n">
-        <v>0.477</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>0.413</v>
+        <v>0.063</v>
       </c>
       <c r="O4" t="n">
-        <v>0.364</v>
+        <v>0.047</v>
       </c>
       <c r="P4" t="n">
-        <v>0.299</v>
+        <v>0.032</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.233</v>
+        <v>0.014</v>
       </c>
       <c r="R4" t="n">
-        <v>0.168</v>
+        <v>0.012</v>
       </c>
       <c r="S4" t="n">
-        <v>0.107</v>
+        <v>0.006</v>
       </c>
       <c r="T4" t="n">
-        <v>0.056</v>
+        <v>0.002</v>
       </c>
       <c r="U4" t="n">
-        <v>0.015</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
         <v>0.001</v>
@@ -1573,68 +1445,68 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>dinov2_ENT</t>
+          <t>inputxgradient</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>0.86</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.624</v>
       </c>
       <c r="D5" t="n">
-        <v>0.798</v>
+        <v>0.513</v>
       </c>
       <c r="E5" t="n">
-        <v>0.769</v>
+        <v>0.423</v>
       </c>
       <c r="F5" t="n">
-        <v>0.768</v>
+        <v>0.348</v>
       </c>
       <c r="G5" t="n">
-        <v>0.731</v>
+        <v>0.286</v>
       </c>
       <c r="H5" t="n">
-        <v>0.7</v>
+        <v>0.25</v>
       </c>
       <c r="I5" t="n">
-        <v>0.652</v>
+        <v>0.213</v>
       </c>
       <c r="J5" t="n">
-        <v>0.618</v>
+        <v>0.184</v>
       </c>
       <c r="K5" t="n">
-        <v>0.571</v>
+        <v>0.142</v>
       </c>
       <c r="L5" t="n">
-        <v>0.515</v>
+        <v>0.118</v>
       </c>
       <c r="M5" t="n">
-        <v>0.472</v>
+        <v>0.096</v>
       </c>
       <c r="N5" t="n">
-        <v>0.412</v>
+        <v>0.077</v>
       </c>
       <c r="O5" t="n">
-        <v>0.366</v>
+        <v>0.058</v>
       </c>
       <c r="P5" t="n">
-        <v>0.311</v>
+        <v>0.041</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.228</v>
+        <v>0.029</v>
       </c>
       <c r="R5" t="n">
-        <v>0.17</v>
+        <v>0.018</v>
       </c>
       <c r="S5" t="n">
-        <v>0.117</v>
+        <v>0.01</v>
       </c>
       <c r="T5" t="n">
-        <v>0.067</v>
+        <v>0.003</v>
       </c>
       <c r="U5" t="n">
-        <v>0.018</v>
+        <v>0</v>
       </c>
       <c r="V5" t="n">
         <v>0.001</v>
@@ -1643,68 +1515,68 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>dinov2_PC1</t>
+          <t>gradientshap</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>0.86</v>
       </c>
       <c r="C6" t="n">
-        <v>0.82</v>
+        <v>0.641</v>
       </c>
       <c r="D6" t="n">
-        <v>0.804</v>
+        <v>0.527</v>
       </c>
       <c r="E6" t="n">
-        <v>0.781</v>
+        <v>0.442</v>
       </c>
       <c r="F6" t="n">
-        <v>0.766</v>
+        <v>0.379</v>
       </c>
       <c r="G6" t="n">
-        <v>0.749</v>
+        <v>0.331</v>
       </c>
       <c r="H6" t="n">
-        <v>0.715</v>
+        <v>0.284</v>
       </c>
       <c r="I6" t="n">
-        <v>0.675</v>
+        <v>0.23</v>
       </c>
       <c r="J6" t="n">
-        <v>0.614</v>
+        <v>0.197</v>
       </c>
       <c r="K6" t="n">
-        <v>0.573</v>
+        <v>0.161</v>
       </c>
       <c r="L6" t="n">
-        <v>0.516</v>
+        <v>0.146</v>
       </c>
       <c r="M6" t="n">
-        <v>0.476</v>
+        <v>0.122</v>
       </c>
       <c r="N6" t="n">
-        <v>0.414</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="O6" t="n">
-        <v>0.344</v>
+        <v>0.076</v>
       </c>
       <c r="P6" t="n">
-        <v>0.299</v>
+        <v>0.056</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.219</v>
+        <v>0.041</v>
       </c>
       <c r="R6" t="n">
-        <v>0.148</v>
+        <v>0.026</v>
       </c>
       <c r="S6" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.015</v>
       </c>
       <c r="T6" t="n">
-        <v>0.043</v>
+        <v>0.006</v>
       </c>
       <c r="U6" t="n">
-        <v>0.014</v>
+        <v>0</v>
       </c>
       <c r="V6" t="n">
         <v>0.001</v>
@@ -1713,68 +1585,68 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dinov2_PC_EV</t>
+          <t>integrated_gradients</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>0.86</v>
       </c>
       <c r="C7" t="n">
-        <v>0.82</v>
+        <v>0.627</v>
       </c>
       <c r="D7" t="n">
-        <v>0.804</v>
+        <v>0.523</v>
       </c>
       <c r="E7" t="n">
-        <v>0.781</v>
+        <v>0.446</v>
       </c>
       <c r="F7" t="n">
-        <v>0.766</v>
+        <v>0.367</v>
       </c>
       <c r="G7" t="n">
-        <v>0.749</v>
+        <v>0.316</v>
       </c>
       <c r="H7" t="n">
-        <v>0.715</v>
+        <v>0.267</v>
       </c>
       <c r="I7" t="n">
-        <v>0.675</v>
+        <v>0.236</v>
       </c>
       <c r="J7" t="n">
-        <v>0.614</v>
+        <v>0.198</v>
       </c>
       <c r="K7" t="n">
-        <v>0.573</v>
+        <v>0.173</v>
       </c>
       <c r="L7" t="n">
-        <v>0.516</v>
+        <v>0.153</v>
       </c>
       <c r="M7" t="n">
-        <v>0.476</v>
+        <v>0.124</v>
       </c>
       <c r="N7" t="n">
-        <v>0.414</v>
+        <v>0.101</v>
       </c>
       <c r="O7" t="n">
-        <v>0.344</v>
+        <v>0.079</v>
       </c>
       <c r="P7" t="n">
-        <v>0.299</v>
+        <v>0.062</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.219</v>
+        <v>0.047</v>
       </c>
       <c r="R7" t="n">
-        <v>0.148</v>
+        <v>0.028</v>
       </c>
       <c r="S7" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.011</v>
       </c>
       <c r="T7" t="n">
-        <v>0.043</v>
+        <v>0.004</v>
       </c>
       <c r="U7" t="n">
-        <v>0.014</v>
+        <v>0</v>
       </c>
       <c r="V7" t="n">
         <v>0.001</v>
@@ -1783,68 +1655,68 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dinov2_PC_L2</t>
+          <t>guided_gradcam</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>0.86</v>
       </c>
       <c r="C8" t="n">
-        <v>0.711</v>
+        <v>0.797</v>
       </c>
       <c r="D8" t="n">
-        <v>0.65</v>
+        <v>0.741</v>
       </c>
       <c r="E8" t="n">
-        <v>0.575</v>
+        <v>0.677</v>
       </c>
       <c r="F8" t="n">
-        <v>0.539</v>
+        <v>0.629</v>
       </c>
       <c r="G8" t="n">
-        <v>0.467</v>
+        <v>0.572</v>
       </c>
       <c r="H8" t="n">
-        <v>0.428</v>
+        <v>0.532</v>
       </c>
       <c r="I8" t="n">
-        <v>0.388</v>
+        <v>0.472</v>
       </c>
       <c r="J8" t="n">
-        <v>0.353</v>
+        <v>0.42</v>
       </c>
       <c r="K8" t="n">
-        <v>0.308</v>
+        <v>0.359</v>
       </c>
       <c r="L8" t="n">
-        <v>0.275</v>
+        <v>0.311</v>
       </c>
       <c r="M8" t="n">
-        <v>0.243</v>
+        <v>0.244</v>
       </c>
       <c r="N8" t="n">
-        <v>0.223</v>
+        <v>0.201</v>
       </c>
       <c r="O8" t="n">
-        <v>0.194</v>
+        <v>0.135</v>
       </c>
       <c r="P8" t="n">
-        <v>0.16</v>
+        <v>0.091</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.136</v>
+        <v>0.064</v>
       </c>
       <c r="R8" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="S8" t="n">
-        <v>0.068</v>
+        <v>0.013</v>
       </c>
       <c r="T8" t="n">
-        <v>0.029</v>
+        <v>0.008</v>
       </c>
       <c r="U8" t="n">
-        <v>0.013</v>
+        <v>0.001</v>
       </c>
       <c r="V8" t="n">
         <v>0.001</v>
@@ -1853,68 +1725,68 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dinov2_attention</t>
+          <t>inputxgradient_continuous</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>0.86</v>
       </c>
       <c r="C9" t="n">
-        <v>0.784</v>
+        <v>0.798</v>
       </c>
       <c r="D9" t="n">
-        <v>0.764</v>
+        <v>0.756</v>
       </c>
       <c r="E9" t="n">
-        <v>0.732</v>
+        <v>0.707</v>
       </c>
       <c r="F9" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.636</v>
       </c>
       <c r="G9" t="n">
-        <v>0.662</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>0.627</v>
+        <v>0.528</v>
       </c>
       <c r="I9" t="n">
-        <v>0.585</v>
+        <v>0.464</v>
       </c>
       <c r="J9" t="n">
-        <v>0.54</v>
+        <v>0.403</v>
       </c>
       <c r="K9" t="n">
-        <v>0.506</v>
+        <v>0.346</v>
       </c>
       <c r="L9" t="n">
-        <v>0.461</v>
+        <v>0.288</v>
       </c>
       <c r="M9" t="n">
-        <v>0.412</v>
+        <v>0.242</v>
       </c>
       <c r="N9" t="n">
-        <v>0.376</v>
+        <v>0.177</v>
       </c>
       <c r="O9" t="n">
-        <v>0.328</v>
+        <v>0.136</v>
       </c>
       <c r="P9" t="n">
-        <v>0.256</v>
+        <v>0.1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.213</v>
+        <v>0.076</v>
       </c>
       <c r="R9" t="n">
-        <v>0.154</v>
+        <v>0.049</v>
       </c>
       <c r="S9" t="n">
-        <v>0.1</v>
+        <v>0.021</v>
       </c>
       <c r="T9" t="n">
-        <v>0.055</v>
+        <v>0.014</v>
       </c>
       <c r="U9" t="n">
-        <v>0.022</v>
+        <v>0.006</v>
       </c>
       <c r="V9" t="n">
         <v>0.001</v>
@@ -1923,68 +1795,68 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>grad_cam</t>
+          <t>xrai</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>0.86</v>
       </c>
       <c r="C10" t="n">
-        <v>0.853</v>
+        <v>0.794</v>
       </c>
       <c r="D10" t="n">
-        <v>0.85</v>
+        <v>0.742</v>
       </c>
       <c r="E10" t="n">
-        <v>0.837</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>0.828</v>
+        <v>0.64</v>
       </c>
       <c r="G10" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.582</v>
       </c>
       <c r="H10" t="n">
-        <v>0.8110000000000001</v>
+        <v>0.521</v>
       </c>
       <c r="I10" t="n">
-        <v>0.801</v>
+        <v>0.478</v>
       </c>
       <c r="J10" t="n">
-        <v>0.783</v>
+        <v>0.397</v>
       </c>
       <c r="K10" t="n">
-        <v>0.755</v>
+        <v>0.36</v>
       </c>
       <c r="L10" t="n">
-        <v>0.75</v>
+        <v>0.321</v>
       </c>
       <c r="M10" t="n">
-        <v>0.699</v>
+        <v>0.274</v>
       </c>
       <c r="N10" t="n">
-        <v>0.663</v>
+        <v>0.212</v>
       </c>
       <c r="O10" t="n">
-        <v>0.62</v>
+        <v>0.171</v>
       </c>
       <c r="P10" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.125</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.494</v>
+        <v>0.091</v>
       </c>
       <c r="R10" t="n">
-        <v>0.405</v>
+        <v>0.062</v>
       </c>
       <c r="S10" t="n">
-        <v>0.276</v>
+        <v>0.038</v>
       </c>
       <c r="T10" t="n">
-        <v>0.124</v>
+        <v>0.019</v>
       </c>
       <c r="U10" t="n">
-        <v>0.028</v>
+        <v>0.005</v>
       </c>
       <c r="V10" t="n">
         <v>0.001</v>
@@ -1993,68 +1865,68 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gradientshap</t>
+          <t>occlusion</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>0.86</v>
       </c>
       <c r="C11" t="n">
-        <v>0.641</v>
+        <v>0.749</v>
       </c>
       <c r="D11" t="n">
-        <v>0.527</v>
+        <v>0.652</v>
       </c>
       <c r="E11" t="n">
-        <v>0.442</v>
+        <v>0.594</v>
       </c>
       <c r="F11" t="n">
-        <v>0.379</v>
+        <v>0.546</v>
       </c>
       <c r="G11" t="n">
-        <v>0.331</v>
+        <v>0.495</v>
       </c>
       <c r="H11" t="n">
-        <v>0.284</v>
+        <v>0.443</v>
       </c>
       <c r="I11" t="n">
-        <v>0.23</v>
+        <v>0.406</v>
       </c>
       <c r="J11" t="n">
-        <v>0.197</v>
+        <v>0.367</v>
       </c>
       <c r="K11" t="n">
-        <v>0.161</v>
+        <v>0.33</v>
       </c>
       <c r="L11" t="n">
-        <v>0.146</v>
+        <v>0.278</v>
       </c>
       <c r="M11" t="n">
-        <v>0.122</v>
+        <v>0.257</v>
       </c>
       <c r="N11" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.218</v>
       </c>
       <c r="O11" t="n">
-        <v>0.076</v>
+        <v>0.186</v>
       </c>
       <c r="P11" t="n">
-        <v>0.056</v>
+        <v>0.155</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.041</v>
+        <v>0.132</v>
       </c>
       <c r="R11" t="n">
-        <v>0.026</v>
+        <v>0.1</v>
       </c>
       <c r="S11" t="n">
-        <v>0.015</v>
+        <v>0.06</v>
       </c>
       <c r="T11" t="n">
-        <v>0.006</v>
+        <v>0.038</v>
       </c>
       <c r="U11" t="n">
-        <v>0</v>
+        <v>0.012</v>
       </c>
       <c r="V11" t="n">
         <v>0.001</v>
@@ -2063,68 +1935,68 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>guided_backprop</t>
+          <t>dinov2_attention</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>0.86</v>
       </c>
       <c r="C12" t="n">
-        <v>0.594</v>
+        <v>0.784</v>
       </c>
       <c r="D12" t="n">
-        <v>0.479</v>
+        <v>0.764</v>
       </c>
       <c r="E12" t="n">
-        <v>0.403</v>
+        <v>0.732</v>
       </c>
       <c r="F12" t="n">
-        <v>0.327</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>0.267</v>
+        <v>0.662</v>
       </c>
       <c r="H12" t="n">
-        <v>0.216</v>
+        <v>0.627</v>
       </c>
       <c r="I12" t="n">
-        <v>0.18</v>
+        <v>0.585</v>
       </c>
       <c r="J12" t="n">
-        <v>0.15</v>
+        <v>0.54</v>
       </c>
       <c r="K12" t="n">
-        <v>0.13</v>
+        <v>0.506</v>
       </c>
       <c r="L12" t="n">
-        <v>0.104</v>
+        <v>0.461</v>
       </c>
       <c r="M12" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.412</v>
       </c>
       <c r="N12" t="n">
-        <v>0.063</v>
+        <v>0.376</v>
       </c>
       <c r="O12" t="n">
-        <v>0.047</v>
+        <v>0.328</v>
       </c>
       <c r="P12" t="n">
-        <v>0.032</v>
+        <v>0.256</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.014</v>
+        <v>0.213</v>
       </c>
       <c r="R12" t="n">
-        <v>0.012</v>
+        <v>0.154</v>
       </c>
       <c r="S12" t="n">
-        <v>0.006</v>
+        <v>0.1</v>
       </c>
       <c r="T12" t="n">
-        <v>0.002</v>
+        <v>0.055</v>
       </c>
       <c r="U12" t="n">
-        <v>0</v>
+        <v>0.022</v>
       </c>
       <c r="V12" t="n">
         <v>0.001</v>
@@ -2133,68 +2005,68 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>guided_gradcam</t>
+          <t>dinov2_PC1</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>0.86</v>
       </c>
       <c r="C13" t="n">
-        <v>0.797</v>
+        <v>0.82</v>
       </c>
       <c r="D13" t="n">
-        <v>0.741</v>
+        <v>0.804</v>
       </c>
       <c r="E13" t="n">
-        <v>0.677</v>
+        <v>0.781</v>
       </c>
       <c r="F13" t="n">
-        <v>0.629</v>
+        <v>0.766</v>
       </c>
       <c r="G13" t="n">
-        <v>0.572</v>
+        <v>0.749</v>
       </c>
       <c r="H13" t="n">
-        <v>0.532</v>
+        <v>0.715</v>
       </c>
       <c r="I13" t="n">
-        <v>0.472</v>
+        <v>0.675</v>
       </c>
       <c r="J13" t="n">
-        <v>0.42</v>
+        <v>0.614</v>
       </c>
       <c r="K13" t="n">
-        <v>0.359</v>
+        <v>0.573</v>
       </c>
       <c r="L13" t="n">
-        <v>0.311</v>
+        <v>0.516</v>
       </c>
       <c r="M13" t="n">
-        <v>0.244</v>
+        <v>0.476</v>
       </c>
       <c r="N13" t="n">
-        <v>0.201</v>
+        <v>0.414</v>
       </c>
       <c r="O13" t="n">
-        <v>0.135</v>
+        <v>0.344</v>
       </c>
       <c r="P13" t="n">
-        <v>0.091</v>
+        <v>0.299</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.064</v>
+        <v>0.219</v>
       </c>
       <c r="R13" t="n">
-        <v>0.04</v>
+        <v>0.148</v>
       </c>
       <c r="S13" t="n">
-        <v>0.013</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="T13" t="n">
-        <v>0.008</v>
+        <v>0.043</v>
       </c>
       <c r="U13" t="n">
-        <v>0.001</v>
+        <v>0.014</v>
       </c>
       <c r="V13" t="n">
         <v>0.001</v>
@@ -2203,68 +2075,68 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>inputxgradient</t>
+          <t>dinov2_COMBO_FIXED</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>0.86</v>
       </c>
       <c r="C14" t="n">
-        <v>0.624</v>
+        <v>0.821</v>
       </c>
       <c r="D14" t="n">
-        <v>0.513</v>
+        <v>0.801</v>
       </c>
       <c r="E14" t="n">
-        <v>0.423</v>
+        <v>0.77</v>
       </c>
       <c r="F14" t="n">
-        <v>0.348</v>
+        <v>0.763</v>
       </c>
       <c r="G14" t="n">
-        <v>0.286</v>
+        <v>0.736</v>
       </c>
       <c r="H14" t="n">
-        <v>0.25</v>
+        <v>0.71</v>
       </c>
       <c r="I14" t="n">
-        <v>0.213</v>
+        <v>0.675</v>
       </c>
       <c r="J14" t="n">
-        <v>0.184</v>
+        <v>0.626</v>
       </c>
       <c r="K14" t="n">
-        <v>0.142</v>
+        <v>0.588</v>
       </c>
       <c r="L14" t="n">
-        <v>0.118</v>
+        <v>0.536</v>
       </c>
       <c r="M14" t="n">
-        <v>0.096</v>
+        <v>0.477</v>
       </c>
       <c r="N14" t="n">
-        <v>0.077</v>
+        <v>0.413</v>
       </c>
       <c r="O14" t="n">
-        <v>0.058</v>
+        <v>0.364</v>
       </c>
       <c r="P14" t="n">
-        <v>0.041</v>
+        <v>0.299</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.029</v>
+        <v>0.233</v>
       </c>
       <c r="R14" t="n">
-        <v>0.018</v>
+        <v>0.168</v>
       </c>
       <c r="S14" t="n">
-        <v>0.01</v>
+        <v>0.107</v>
       </c>
       <c r="T14" t="n">
-        <v>0.003</v>
+        <v>0.056</v>
       </c>
       <c r="U14" t="n">
-        <v>0</v>
+        <v>0.015</v>
       </c>
       <c r="V14" t="n">
         <v>0.001</v>
@@ -2273,68 +2145,68 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>inputxgradient_continuous</t>
+          <t>u2net_dino_fusion</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>0.86</v>
       </c>
       <c r="C15" t="n">
-        <v>0.798</v>
+        <v>0.804</v>
       </c>
       <c r="D15" t="n">
-        <v>0.756</v>
+        <v>0.795</v>
       </c>
       <c r="E15" t="n">
-        <v>0.707</v>
+        <v>0.773</v>
       </c>
       <c r="F15" t="n">
-        <v>0.636</v>
+        <v>0.755</v>
       </c>
       <c r="G15" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.723</v>
       </c>
       <c r="H15" t="n">
-        <v>0.528</v>
+        <v>0.712</v>
       </c>
       <c r="I15" t="n">
-        <v>0.464</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>0.403</v>
+        <v>0.645</v>
       </c>
       <c r="K15" t="n">
-        <v>0.346</v>
+        <v>0.625</v>
       </c>
       <c r="L15" t="n">
-        <v>0.288</v>
+        <v>0.585</v>
       </c>
       <c r="M15" t="n">
-        <v>0.242</v>
+        <v>0.536</v>
       </c>
       <c r="N15" t="n">
-        <v>0.177</v>
+        <v>0.498</v>
       </c>
       <c r="O15" t="n">
-        <v>0.136</v>
+        <v>0.437</v>
       </c>
       <c r="P15" t="n">
-        <v>0.1</v>
+        <v>0.371</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.076</v>
+        <v>0.297</v>
       </c>
       <c r="R15" t="n">
-        <v>0.049</v>
+        <v>0.232</v>
       </c>
       <c r="S15" t="n">
-        <v>0.021</v>
+        <v>0.15</v>
       </c>
       <c r="T15" t="n">
-        <v>0.014</v>
+        <v>0.089</v>
       </c>
       <c r="U15" t="n">
-        <v>0.006</v>
+        <v>0.033</v>
       </c>
       <c r="V15" t="n">
         <v>0.001</v>
@@ -2343,68 +2215,68 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>inputxgradient_u2net_fill</t>
+          <t>U2Net-Saliency</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>0.86</v>
       </c>
       <c r="C16" t="n">
-        <v>0.757</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>0.716</v>
+        <v>0.797</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.764</v>
       </c>
       <c r="F16" t="n">
-        <v>0.674</v>
+        <v>0.754</v>
       </c>
       <c r="G16" t="n">
-        <v>0.646</v>
+        <v>0.755</v>
       </c>
       <c r="H16" t="n">
-        <v>0.615</v>
+        <v>0.741</v>
       </c>
       <c r="I16" t="n">
-        <v>0.594</v>
+        <v>0.712</v>
       </c>
       <c r="J16" t="n">
+        <v>0.6830000000000001</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.666</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.608</v>
+      </c>
+      <c r="M16" t="n">
         <v>0.5659999999999999</v>
       </c>
-      <c r="K16" t="n">
-        <v>0.538</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0.527</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0.502</v>
-      </c>
       <c r="N16" t="n">
-        <v>0.456</v>
+        <v>0.519</v>
       </c>
       <c r="O16" t="n">
-        <v>0.421</v>
+        <v>0.465</v>
       </c>
       <c r="P16" t="n">
-        <v>0.365</v>
+        <v>0.395</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.324</v>
+        <v>0.31</v>
       </c>
       <c r="R16" t="n">
-        <v>0.246</v>
+        <v>0.237</v>
       </c>
       <c r="S16" t="n">
-        <v>0.183</v>
+        <v>0.151</v>
       </c>
       <c r="T16" t="n">
-        <v>0.091</v>
+        <v>0.081</v>
       </c>
       <c r="U16" t="n">
-        <v>0.032</v>
+        <v>0.036</v>
       </c>
       <c r="V16" t="n">
         <v>0.001</v>
@@ -2413,68 +2285,68 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>integrated_gradients</t>
+          <t>inputxgradient_u2net_fill</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>0.86</v>
       </c>
       <c r="C17" t="n">
-        <v>0.627</v>
+        <v>0.757</v>
       </c>
       <c r="D17" t="n">
-        <v>0.523</v>
+        <v>0.716</v>
       </c>
       <c r="E17" t="n">
-        <v>0.446</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>0.367</v>
+        <v>0.674</v>
       </c>
       <c r="G17" t="n">
-        <v>0.316</v>
+        <v>0.646</v>
       </c>
       <c r="H17" t="n">
-        <v>0.267</v>
+        <v>0.615</v>
       </c>
       <c r="I17" t="n">
-        <v>0.236</v>
+        <v>0.594</v>
       </c>
       <c r="J17" t="n">
-        <v>0.198</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="K17" t="n">
-        <v>0.173</v>
+        <v>0.538</v>
       </c>
       <c r="L17" t="n">
-        <v>0.153</v>
+        <v>0.527</v>
       </c>
       <c r="M17" t="n">
-        <v>0.124</v>
+        <v>0.502</v>
       </c>
       <c r="N17" t="n">
-        <v>0.101</v>
+        <v>0.456</v>
       </c>
       <c r="O17" t="n">
-        <v>0.079</v>
+        <v>0.421</v>
       </c>
       <c r="P17" t="n">
-        <v>0.062</v>
+        <v>0.365</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.047</v>
+        <v>0.324</v>
       </c>
       <c r="R17" t="n">
-        <v>0.028</v>
+        <v>0.246</v>
       </c>
       <c r="S17" t="n">
-        <v>0.011</v>
+        <v>0.183</v>
       </c>
       <c r="T17" t="n">
-        <v>0.004</v>
+        <v>0.091</v>
       </c>
       <c r="U17" t="n">
-        <v>0</v>
+        <v>0.032</v>
       </c>
       <c r="V17" t="n">
         <v>0.001</v>
@@ -2483,68 +2355,68 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>occlusion</t>
+          <t>dinov2_COMBO_ENT_SMOOTH</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>0.86</v>
       </c>
       <c r="C18" t="n">
-        <v>0.749</v>
+        <v>0.852</v>
       </c>
       <c r="D18" t="n">
-        <v>0.652</v>
+        <v>0.83</v>
       </c>
       <c r="E18" t="n">
-        <v>0.594</v>
+        <v>0.826</v>
       </c>
       <c r="F18" t="n">
-        <v>0.546</v>
+        <v>0.805</v>
       </c>
       <c r="G18" t="n">
-        <v>0.495</v>
+        <v>0.796</v>
       </c>
       <c r="H18" t="n">
-        <v>0.443</v>
+        <v>0.774</v>
       </c>
       <c r="I18" t="n">
-        <v>0.406</v>
+        <v>0.756</v>
       </c>
       <c r="J18" t="n">
+        <v>0.723</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.694</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.5659999999999999</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.518</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="Q18" t="n">
         <v>0.367</v>
       </c>
-      <c r="K18" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0.278</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0.257</v>
-      </c>
-      <c r="N18" t="n">
-        <v>0.218</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0.186</v>
-      </c>
-      <c r="P18" t="n">
-        <v>0.155</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>0.132</v>
-      </c>
       <c r="R18" t="n">
-        <v>0.1</v>
+        <v>0.295</v>
       </c>
       <c r="S18" t="n">
-        <v>0.06</v>
+        <v>0.212</v>
       </c>
       <c r="T18" t="n">
-        <v>0.038</v>
+        <v>0.123</v>
       </c>
       <c r="U18" t="n">
-        <v>0.012</v>
+        <v>0.051</v>
       </c>
       <c r="V18" t="n">
         <v>0.001</v>
@@ -2553,354 +2425,86 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>random_baseline</t>
+          <t>grad_cam</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>0.86</v>
       </c>
       <c r="C19" t="n">
-        <v>0.379</v>
+        <v>0.853</v>
       </c>
       <c r="D19" t="n">
-        <v>0.307</v>
+        <v>0.85</v>
       </c>
       <c r="E19" t="n">
-        <v>0.221</v>
+        <v>0.837</v>
       </c>
       <c r="F19" t="n">
-        <v>0.154</v>
+        <v>0.828</v>
       </c>
       <c r="G19" t="n">
-        <v>0.109</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>0.079</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>0.054</v>
+        <v>0.801</v>
       </c>
       <c r="J19" t="n">
-        <v>0.046</v>
+        <v>0.783</v>
       </c>
       <c r="K19" t="n">
-        <v>0.032</v>
+        <v>0.755</v>
       </c>
       <c r="L19" t="n">
-        <v>0.024</v>
+        <v>0.75</v>
       </c>
       <c r="M19" t="n">
-        <v>0.022</v>
+        <v>0.699</v>
       </c>
       <c r="N19" t="n">
-        <v>0.014</v>
+        <v>0.663</v>
       </c>
       <c r="O19" t="n">
-        <v>0.012</v>
+        <v>0.62</v>
       </c>
       <c r="P19" t="n">
-        <v>0.008</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.005</v>
+        <v>0.494</v>
       </c>
       <c r="R19" t="n">
-        <v>0.001</v>
+        <v>0.405</v>
       </c>
       <c r="S19" t="n">
-        <v>0.003</v>
+        <v>0.276</v>
       </c>
       <c r="T19" t="n">
-        <v>0</v>
+        <v>0.124</v>
       </c>
       <c r="U19" t="n">
-        <v>0.001</v>
+        <v>0.028</v>
       </c>
       <c r="V19" t="n">
         <v>0.001</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>saliency</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0.597</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0.478</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.408</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0.322</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.263</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.219</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0.177</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0.145</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0.104</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.074</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="O20" t="n">
-        <v>0.046</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="R20" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="S20" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="T20" t="n">
-        <v>0.003</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>sumDino</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.8169999999999999</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0.786</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.759</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.742</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.717</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0.671</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0.617</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.579</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0.524</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0.472</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.439</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0.366</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0.296</v>
-      </c>
-      <c r="P21" t="n">
-        <v>0.247</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="R21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="S21" t="n">
-        <v>0.093</v>
-      </c>
-      <c r="T21" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="U21" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="V21" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>u2net_dino_fusion</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0.8129999999999999</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.776</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0.736</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0.714</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0.699</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.654</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0.591</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.537</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0.481</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0.418</v>
-      </c>
-      <c r="P22" t="n">
-        <v>0.383</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0.324</v>
-      </c>
-      <c r="R22" t="n">
-        <v>0.235</v>
-      </c>
-      <c r="S22" t="n">
-        <v>0.165</v>
-      </c>
-      <c r="T22" t="n">
-        <v>0.079</v>
-      </c>
-      <c r="U22" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="V22" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>xrai</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.794</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0.742</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0.582</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.521</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0.478</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.397</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0.321</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0.274</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.212</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0.171</v>
-      </c>
-      <c r="P23" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="R23" t="n">
-        <v>0.062</v>
-      </c>
-      <c r="S23" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="T23" t="n">
-        <v>0.019</v>
-      </c>
-      <c r="U23" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="V23" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:V19">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed the crop in loader.py optimize phase2_runner.py and refactor a little
</commit_message>
<xml_diff>
--- a/results/excel_reports/mobilenet_v2_resnet50_black.xlsx
+++ b/results/excel_reports/mobilenet_v2_resnet50_black.xlsx
@@ -656,102 +656,6 @@
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="15"/>
-          <order val="15"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A17</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$17:$V$17</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="16"/>
-          <order val="16"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A18</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$18:$V$18</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="17"/>
-          <order val="17"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A19</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$19:$V$19</f>
-            </numRef>
-          </val>
-        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -825,7 +729,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>21</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9000000" cy="5400000"/>
@@ -1135,11 +1039,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -1239,61 +1143,61 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C2" t="n">
-        <v>0.379</v>
+        <v>0.365</v>
       </c>
       <c r="D2" t="n">
-        <v>0.307</v>
+        <v>0.254</v>
       </c>
       <c r="E2" t="n">
-        <v>0.221</v>
+        <v>0.156</v>
       </c>
       <c r="F2" t="n">
-        <v>0.154</v>
+        <v>0.096</v>
       </c>
       <c r="G2" t="n">
-        <v>0.109</v>
+        <v>0.063</v>
       </c>
       <c r="H2" t="n">
-        <v>0.079</v>
+        <v>0.044</v>
       </c>
       <c r="I2" t="n">
-        <v>0.054</v>
+        <v>0.028</v>
       </c>
       <c r="J2" t="n">
-        <v>0.046</v>
+        <v>0.024</v>
       </c>
       <c r="K2" t="n">
-        <v>0.032</v>
+        <v>0.013</v>
       </c>
       <c r="L2" t="n">
-        <v>0.024</v>
+        <v>0.011</v>
       </c>
       <c r="M2" t="n">
-        <v>0.022</v>
+        <v>0.01</v>
       </c>
       <c r="N2" t="n">
-        <v>0.014</v>
+        <v>0.008</v>
       </c>
       <c r="O2" t="n">
-        <v>0.012</v>
+        <v>0.006</v>
       </c>
       <c r="P2" t="n">
-        <v>0.008</v>
+        <v>0.005</v>
       </c>
       <c r="Q2" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="R2" t="n">
         <v>0.005</v>
       </c>
-      <c r="R2" t="n">
-        <v>0.001</v>
-      </c>
       <c r="S2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="T2" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="U2" t="n">
         <v>0.001</v>
@@ -1305,65 +1209,65 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>saliency</t>
+          <t>guided_backprop</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C3" t="n">
-        <v>0.597</v>
+        <v>0.586</v>
       </c>
       <c r="D3" t="n">
-        <v>0.478</v>
+        <v>0.463</v>
       </c>
       <c r="E3" t="n">
-        <v>0.408</v>
+        <v>0.378</v>
       </c>
       <c r="F3" t="n">
-        <v>0.322</v>
+        <v>0.306</v>
       </c>
       <c r="G3" t="n">
-        <v>0.263</v>
+        <v>0.235</v>
       </c>
       <c r="H3" t="n">
-        <v>0.219</v>
+        <v>0.193</v>
       </c>
       <c r="I3" t="n">
-        <v>0.177</v>
+        <v>0.141</v>
       </c>
       <c r="J3" t="n">
-        <v>0.145</v>
+        <v>0.117</v>
       </c>
       <c r="K3" t="n">
-        <v>0.13</v>
+        <v>0.089</v>
       </c>
       <c r="L3" t="n">
-        <v>0.104</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>0.074</v>
+        <v>0.055</v>
       </c>
       <c r="N3" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="O3" t="n">
-        <v>0.046</v>
+        <v>0.03</v>
       </c>
       <c r="P3" t="n">
-        <v>0.028</v>
+        <v>0.014</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.014</v>
+        <v>0.013</v>
       </c>
       <c r="R3" t="n">
-        <v>0.01</v>
+        <v>0.008</v>
       </c>
       <c r="S3" t="n">
-        <v>0.006</v>
+        <v>0.002</v>
       </c>
       <c r="T3" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -1375,65 +1279,65 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>guided_backprop</t>
+          <t>saliency</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C4" t="n">
-        <v>0.594</v>
+        <v>0.583</v>
       </c>
       <c r="D4" t="n">
-        <v>0.479</v>
+        <v>0.46</v>
       </c>
       <c r="E4" t="n">
-        <v>0.403</v>
+        <v>0.375</v>
       </c>
       <c r="F4" t="n">
-        <v>0.327</v>
+        <v>0.304</v>
       </c>
       <c r="G4" t="n">
-        <v>0.267</v>
+        <v>0.238</v>
       </c>
       <c r="H4" t="n">
-        <v>0.216</v>
+        <v>0.198</v>
       </c>
       <c r="I4" t="n">
-        <v>0.18</v>
+        <v>0.153</v>
       </c>
       <c r="J4" t="n">
-        <v>0.15</v>
+        <v>0.118</v>
       </c>
       <c r="K4" t="n">
-        <v>0.13</v>
+        <v>0.091</v>
       </c>
       <c r="L4" t="n">
-        <v>0.104</v>
+        <v>0.074</v>
       </c>
       <c r="M4" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.05</v>
       </c>
       <c r="N4" t="n">
-        <v>0.063</v>
+        <v>0.039</v>
       </c>
       <c r="O4" t="n">
-        <v>0.047</v>
+        <v>0.03</v>
       </c>
       <c r="P4" t="n">
-        <v>0.032</v>
+        <v>0.017</v>
       </c>
       <c r="Q4" t="n">
         <v>0.014</v>
       </c>
       <c r="R4" t="n">
-        <v>0.012</v>
+        <v>0.006</v>
       </c>
       <c r="S4" t="n">
-        <v>0.006</v>
+        <v>0.003</v>
       </c>
       <c r="T4" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -1449,61 +1353,61 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C5" t="n">
-        <v>0.624</v>
+        <v>0.576</v>
       </c>
       <c r="D5" t="n">
-        <v>0.513</v>
+        <v>0.448</v>
       </c>
       <c r="E5" t="n">
-        <v>0.423</v>
+        <v>0.354</v>
       </c>
       <c r="F5" t="n">
-        <v>0.348</v>
+        <v>0.277</v>
       </c>
       <c r="G5" t="n">
-        <v>0.286</v>
+        <v>0.243</v>
       </c>
       <c r="H5" t="n">
-        <v>0.25</v>
+        <v>0.199</v>
       </c>
       <c r="I5" t="n">
-        <v>0.213</v>
+        <v>0.159</v>
       </c>
       <c r="J5" t="n">
-        <v>0.184</v>
+        <v>0.123</v>
       </c>
       <c r="K5" t="n">
-        <v>0.142</v>
+        <v>0.109</v>
       </c>
       <c r="L5" t="n">
-        <v>0.118</v>
+        <v>0.093</v>
       </c>
       <c r="M5" t="n">
-        <v>0.096</v>
+        <v>0.059</v>
       </c>
       <c r="N5" t="n">
-        <v>0.077</v>
+        <v>0.048</v>
       </c>
       <c r="O5" t="n">
-        <v>0.058</v>
+        <v>0.039</v>
       </c>
       <c r="P5" t="n">
-        <v>0.041</v>
+        <v>0.022</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.029</v>
+        <v>0.018</v>
       </c>
       <c r="R5" t="n">
-        <v>0.018</v>
+        <v>0.01</v>
       </c>
       <c r="S5" t="n">
-        <v>0.01</v>
+        <v>0.004</v>
       </c>
       <c r="T5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -1519,61 +1423,61 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C6" t="n">
-        <v>0.641</v>
+        <v>0.588</v>
       </c>
       <c r="D6" t="n">
-        <v>0.527</v>
+        <v>0.48</v>
       </c>
       <c r="E6" t="n">
-        <v>0.442</v>
+        <v>0.398</v>
       </c>
       <c r="F6" t="n">
-        <v>0.379</v>
+        <v>0.321</v>
       </c>
       <c r="G6" t="n">
-        <v>0.331</v>
+        <v>0.276</v>
       </c>
       <c r="H6" t="n">
-        <v>0.284</v>
+        <v>0.22</v>
       </c>
       <c r="I6" t="n">
-        <v>0.23</v>
+        <v>0.187</v>
       </c>
       <c r="J6" t="n">
-        <v>0.197</v>
+        <v>0.158</v>
       </c>
       <c r="K6" t="n">
-        <v>0.161</v>
+        <v>0.137</v>
       </c>
       <c r="L6" t="n">
-        <v>0.146</v>
+        <v>0.099</v>
       </c>
       <c r="M6" t="n">
-        <v>0.122</v>
+        <v>0.079</v>
       </c>
       <c r="N6" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.059</v>
       </c>
       <c r="O6" t="n">
-        <v>0.076</v>
+        <v>0.037</v>
       </c>
       <c r="P6" t="n">
-        <v>0.056</v>
+        <v>0.029</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.041</v>
+        <v>0.021</v>
       </c>
       <c r="R6" t="n">
-        <v>0.026</v>
+        <v>0.016</v>
       </c>
       <c r="S6" t="n">
-        <v>0.015</v>
+        <v>0.007</v>
       </c>
       <c r="T6" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -1589,61 +1493,61 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C7" t="n">
-        <v>0.627</v>
+        <v>0.609</v>
       </c>
       <c r="D7" t="n">
-        <v>0.523</v>
+        <v>0.49</v>
       </c>
       <c r="E7" t="n">
-        <v>0.446</v>
+        <v>0.41</v>
       </c>
       <c r="F7" t="n">
-        <v>0.367</v>
+        <v>0.33</v>
       </c>
       <c r="G7" t="n">
-        <v>0.316</v>
+        <v>0.272</v>
       </c>
       <c r="H7" t="n">
-        <v>0.267</v>
+        <v>0.215</v>
       </c>
       <c r="I7" t="n">
-        <v>0.236</v>
+        <v>0.188</v>
       </c>
       <c r="J7" t="n">
-        <v>0.198</v>
+        <v>0.156</v>
       </c>
       <c r="K7" t="n">
-        <v>0.173</v>
+        <v>0.133</v>
       </c>
       <c r="L7" t="n">
-        <v>0.153</v>
+        <v>0.108</v>
       </c>
       <c r="M7" t="n">
-        <v>0.124</v>
+        <v>0.091</v>
       </c>
       <c r="N7" t="n">
-        <v>0.101</v>
+        <v>0.058</v>
       </c>
       <c r="O7" t="n">
-        <v>0.079</v>
+        <v>0.044</v>
       </c>
       <c r="P7" t="n">
-        <v>0.062</v>
+        <v>0.026</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.047</v>
+        <v>0.022</v>
       </c>
       <c r="R7" t="n">
-        <v>0.028</v>
+        <v>0.014</v>
       </c>
       <c r="S7" t="n">
-        <v>0.011</v>
+        <v>0.007</v>
       </c>
       <c r="T7" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -1659,61 +1563,61 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C8" t="n">
-        <v>0.797</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>0.741</v>
+        <v>0.748</v>
       </c>
       <c r="E8" t="n">
-        <v>0.677</v>
+        <v>0.721</v>
       </c>
       <c r="F8" t="n">
-        <v>0.629</v>
+        <v>0.664</v>
       </c>
       <c r="G8" t="n">
-        <v>0.572</v>
+        <v>0.614</v>
       </c>
       <c r="H8" t="n">
-        <v>0.532</v>
+        <v>0.547</v>
       </c>
       <c r="I8" t="n">
-        <v>0.472</v>
+        <v>0.475</v>
       </c>
       <c r="J8" t="n">
-        <v>0.42</v>
+        <v>0.418</v>
       </c>
       <c r="K8" t="n">
-        <v>0.359</v>
+        <v>0.361</v>
       </c>
       <c r="L8" t="n">
-        <v>0.311</v>
+        <v>0.292</v>
       </c>
       <c r="M8" t="n">
         <v>0.244</v>
       </c>
       <c r="N8" t="n">
-        <v>0.201</v>
+        <v>0.189</v>
       </c>
       <c r="O8" t="n">
-        <v>0.135</v>
+        <v>0.139</v>
       </c>
       <c r="P8" t="n">
-        <v>0.091</v>
+        <v>0.093</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.064</v>
+        <v>0.061</v>
       </c>
       <c r="R8" t="n">
-        <v>0.04</v>
+        <v>0.028</v>
       </c>
       <c r="S8" t="n">
-        <v>0.013</v>
+        <v>0.011</v>
       </c>
       <c r="T8" t="n">
-        <v>0.008</v>
+        <v>0.002</v>
       </c>
       <c r="U8" t="n">
         <v>0.001</v>
@@ -1725,65 +1629,65 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>inputxgradient_continuous</t>
+          <t>xrai</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C9" t="n">
-        <v>0.798</v>
+        <v>0.791</v>
       </c>
       <c r="D9" t="n">
-        <v>0.756</v>
+        <v>0.74</v>
       </c>
       <c r="E9" t="n">
-        <v>0.707</v>
+        <v>0.697</v>
       </c>
       <c r="F9" t="n">
-        <v>0.636</v>
+        <v>0.642</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.586</v>
       </c>
       <c r="H9" t="n">
-        <v>0.528</v>
+        <v>0.529</v>
       </c>
       <c r="I9" t="n">
-        <v>0.464</v>
+        <v>0.481</v>
       </c>
       <c r="J9" t="n">
-        <v>0.403</v>
+        <v>0.432</v>
       </c>
       <c r="K9" t="n">
-        <v>0.346</v>
+        <v>0.384</v>
       </c>
       <c r="L9" t="n">
-        <v>0.288</v>
+        <v>0.333</v>
       </c>
       <c r="M9" t="n">
-        <v>0.242</v>
+        <v>0.291</v>
       </c>
       <c r="N9" t="n">
-        <v>0.177</v>
+        <v>0.246</v>
       </c>
       <c r="O9" t="n">
-        <v>0.136</v>
+        <v>0.202</v>
       </c>
       <c r="P9" t="n">
-        <v>0.1</v>
+        <v>0.153</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.076</v>
+        <v>0.099</v>
       </c>
       <c r="R9" t="n">
-        <v>0.049</v>
+        <v>0.064</v>
       </c>
       <c r="S9" t="n">
-        <v>0.021</v>
+        <v>0.032</v>
       </c>
       <c r="T9" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
       <c r="U9" t="n">
         <v>0.006</v>
@@ -1795,68 +1699,68 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>xrai</t>
+          <t>occlusion</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C10" t="n">
-        <v>0.794</v>
+        <v>0.746</v>
       </c>
       <c r="D10" t="n">
-        <v>0.742</v>
+        <v>0.661</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.603</v>
       </c>
       <c r="F10" t="n">
-        <v>0.64</v>
+        <v>0.535</v>
       </c>
       <c r="G10" t="n">
-        <v>0.582</v>
+        <v>0.482</v>
       </c>
       <c r="H10" t="n">
-        <v>0.521</v>
+        <v>0.456</v>
       </c>
       <c r="I10" t="n">
-        <v>0.478</v>
+        <v>0.409</v>
       </c>
       <c r="J10" t="n">
-        <v>0.397</v>
+        <v>0.37</v>
       </c>
       <c r="K10" t="n">
-        <v>0.36</v>
+        <v>0.346</v>
       </c>
       <c r="L10" t="n">
-        <v>0.321</v>
+        <v>0.311</v>
       </c>
       <c r="M10" t="n">
-        <v>0.274</v>
+        <v>0.269</v>
       </c>
       <c r="N10" t="n">
-        <v>0.212</v>
+        <v>0.23</v>
       </c>
       <c r="O10" t="n">
-        <v>0.171</v>
+        <v>0.204</v>
       </c>
       <c r="P10" t="n">
-        <v>0.125</v>
+        <v>0.181</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.091</v>
+        <v>0.134</v>
       </c>
       <c r="R10" t="n">
-        <v>0.062</v>
+        <v>0.104</v>
       </c>
       <c r="S10" t="n">
-        <v>0.038</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="T10" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="U10" t="n">
         <v>0.019</v>
-      </c>
-      <c r="U10" t="n">
-        <v>0.005</v>
       </c>
       <c r="V10" t="n">
         <v>0.001</v>
@@ -1865,68 +1769,68 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>occlusion</t>
+          <t>dinov2_attention</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C11" t="n">
-        <v>0.749</v>
+        <v>0.804</v>
       </c>
       <c r="D11" t="n">
-        <v>0.652</v>
+        <v>0.778</v>
       </c>
       <c r="E11" t="n">
-        <v>0.594</v>
+        <v>0.745</v>
       </c>
       <c r="F11" t="n">
-        <v>0.546</v>
+        <v>0.727</v>
       </c>
       <c r="G11" t="n">
-        <v>0.495</v>
+        <v>0.699</v>
       </c>
       <c r="H11" t="n">
-        <v>0.443</v>
+        <v>0.676</v>
       </c>
       <c r="I11" t="n">
-        <v>0.406</v>
+        <v>0.641</v>
       </c>
       <c r="J11" t="n">
-        <v>0.367</v>
+        <v>0.599</v>
       </c>
       <c r="K11" t="n">
-        <v>0.33</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>0.278</v>
+        <v>0.521</v>
       </c>
       <c r="M11" t="n">
-        <v>0.257</v>
+        <v>0.491</v>
       </c>
       <c r="N11" t="n">
-        <v>0.218</v>
+        <v>0.445</v>
       </c>
       <c r="O11" t="n">
-        <v>0.186</v>
+        <v>0.394</v>
       </c>
       <c r="P11" t="n">
-        <v>0.155</v>
+        <v>0.333</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.132</v>
+        <v>0.27</v>
       </c>
       <c r="R11" t="n">
-        <v>0.1</v>
+        <v>0.195</v>
       </c>
       <c r="S11" t="n">
-        <v>0.06</v>
+        <v>0.147</v>
       </c>
       <c r="T11" t="n">
-        <v>0.038</v>
+        <v>0.066</v>
       </c>
       <c r="U11" t="n">
-        <v>0.012</v>
+        <v>0.03</v>
       </c>
       <c r="V11" t="n">
         <v>0.001</v>
@@ -1935,68 +1839,68 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dinov2_attention</t>
+          <t>u2net_dino_product</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C12" t="n">
-        <v>0.784</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="D12" t="n">
-        <v>0.764</v>
+        <v>0.785</v>
       </c>
       <c r="E12" t="n">
-        <v>0.732</v>
+        <v>0.76</v>
       </c>
       <c r="F12" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.739</v>
       </c>
       <c r="G12" t="n">
-        <v>0.662</v>
+        <v>0.712</v>
       </c>
       <c r="H12" t="n">
-        <v>0.627</v>
+        <v>0.718</v>
       </c>
       <c r="I12" t="n">
-        <v>0.585</v>
+        <v>0.681</v>
       </c>
       <c r="J12" t="n">
-        <v>0.54</v>
+        <v>0.663</v>
       </c>
       <c r="K12" t="n">
-        <v>0.506</v>
+        <v>0.629</v>
       </c>
       <c r="L12" t="n">
-        <v>0.461</v>
+        <v>0.587</v>
       </c>
       <c r="M12" t="n">
-        <v>0.412</v>
+        <v>0.55</v>
       </c>
       <c r="N12" t="n">
-        <v>0.376</v>
+        <v>0.499</v>
       </c>
       <c r="O12" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.394</v>
+      </c>
+      <c r="Q12" t="n">
         <v>0.328</v>
       </c>
-      <c r="P12" t="n">
-        <v>0.256</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0.213</v>
-      </c>
       <c r="R12" t="n">
-        <v>0.154</v>
+        <v>0.235</v>
       </c>
       <c r="S12" t="n">
-        <v>0.1</v>
+        <v>0.17</v>
       </c>
       <c r="T12" t="n">
-        <v>0.055</v>
+        <v>0.099</v>
       </c>
       <c r="U12" t="n">
-        <v>0.022</v>
+        <v>0.038</v>
       </c>
       <c r="V12" t="n">
         <v>0.001</v>
@@ -2005,68 +1909,68 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dinov2_PC1</t>
+          <t>u2net_dino_fusion</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C13" t="n">
-        <v>0.82</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="D13" t="n">
-        <v>0.804</v>
+        <v>0.782</v>
       </c>
       <c r="E13" t="n">
-        <v>0.781</v>
+        <v>0.752</v>
       </c>
       <c r="F13" t="n">
-        <v>0.766</v>
+        <v>0.733</v>
       </c>
       <c r="G13" t="n">
-        <v>0.749</v>
+        <v>0.713</v>
       </c>
       <c r="H13" t="n">
-        <v>0.715</v>
+        <v>0.7</v>
       </c>
       <c r="I13" t="n">
-        <v>0.675</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>0.614</v>
+        <v>0.659</v>
       </c>
       <c r="K13" t="n">
-        <v>0.573</v>
+        <v>0.618</v>
       </c>
       <c r="L13" t="n">
-        <v>0.516</v>
+        <v>0.591</v>
       </c>
       <c r="M13" t="n">
-        <v>0.476</v>
+        <v>0.554</v>
       </c>
       <c r="N13" t="n">
-        <v>0.414</v>
+        <v>0.513</v>
       </c>
       <c r="O13" t="n">
-        <v>0.344</v>
+        <v>0.459</v>
       </c>
       <c r="P13" t="n">
-        <v>0.299</v>
+        <v>0.401</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.219</v>
+        <v>0.339</v>
       </c>
       <c r="R13" t="n">
-        <v>0.148</v>
+        <v>0.249</v>
       </c>
       <c r="S13" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.168</v>
       </c>
       <c r="T13" t="n">
-        <v>0.043</v>
+        <v>0.097</v>
       </c>
       <c r="U13" t="n">
-        <v>0.014</v>
+        <v>0.04</v>
       </c>
       <c r="V13" t="n">
         <v>0.001</v>
@@ -2075,68 +1979,68 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dinov2_COMBO_FIXED</t>
+          <t>U2Net-Saliency</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C14" t="n">
-        <v>0.821</v>
+        <v>0.839</v>
       </c>
       <c r="D14" t="n">
-        <v>0.801</v>
+        <v>0.833</v>
       </c>
       <c r="E14" t="n">
-        <v>0.77</v>
+        <v>0.82</v>
       </c>
       <c r="F14" t="n">
-        <v>0.763</v>
+        <v>0.802</v>
       </c>
       <c r="G14" t="n">
-        <v>0.736</v>
+        <v>0.786</v>
       </c>
       <c r="H14" t="n">
-        <v>0.71</v>
+        <v>0.767</v>
       </c>
       <c r="I14" t="n">
-        <v>0.675</v>
+        <v>0.731</v>
       </c>
       <c r="J14" t="n">
-        <v>0.626</v>
+        <v>0.704</v>
       </c>
       <c r="K14" t="n">
-        <v>0.588</v>
+        <v>0.673</v>
       </c>
       <c r="L14" t="n">
-        <v>0.536</v>
+        <v>0.634</v>
       </c>
       <c r="M14" t="n">
-        <v>0.477</v>
+        <v>0.58</v>
       </c>
       <c r="N14" t="n">
-        <v>0.413</v>
+        <v>0.542</v>
       </c>
       <c r="O14" t="n">
-        <v>0.364</v>
+        <v>0.496</v>
       </c>
       <c r="P14" t="n">
-        <v>0.299</v>
+        <v>0.443</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.233</v>
+        <v>0.363</v>
       </c>
       <c r="R14" t="n">
-        <v>0.168</v>
+        <v>0.291</v>
       </c>
       <c r="S14" t="n">
-        <v>0.107</v>
+        <v>0.199</v>
       </c>
       <c r="T14" t="n">
-        <v>0.056</v>
+        <v>0.115</v>
       </c>
       <c r="U14" t="n">
-        <v>0.015</v>
+        <v>0.04</v>
       </c>
       <c r="V14" t="n">
         <v>0.001</v>
@@ -2145,68 +2049,68 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>u2net_dino_fusion</t>
+          <t>dinov2_COMBO_ENT_SMOOTH</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C15" t="n">
-        <v>0.804</v>
+        <v>0.844</v>
       </c>
       <c r="D15" t="n">
-        <v>0.795</v>
+        <v>0.832</v>
       </c>
       <c r="E15" t="n">
-        <v>0.773</v>
+        <v>0.826</v>
       </c>
       <c r="F15" t="n">
-        <v>0.755</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>0.723</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>0.712</v>
+        <v>0.797</v>
       </c>
       <c r="I15" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.763</v>
       </c>
       <c r="J15" t="n">
-        <v>0.645</v>
+        <v>0.741</v>
       </c>
       <c r="K15" t="n">
-        <v>0.625</v>
+        <v>0.716</v>
       </c>
       <c r="L15" t="n">
-        <v>0.585</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="M15" t="n">
-        <v>0.536</v>
+        <v>0.656</v>
       </c>
       <c r="N15" t="n">
-        <v>0.498</v>
+        <v>0.595</v>
       </c>
       <c r="O15" t="n">
-        <v>0.437</v>
+        <v>0.541</v>
       </c>
       <c r="P15" t="n">
-        <v>0.371</v>
+        <v>0.495</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.297</v>
+        <v>0.417</v>
       </c>
       <c r="R15" t="n">
-        <v>0.232</v>
+        <v>0.322</v>
       </c>
       <c r="S15" t="n">
-        <v>0.15</v>
+        <v>0.207</v>
       </c>
       <c r="T15" t="n">
-        <v>0.089</v>
+        <v>0.111</v>
       </c>
       <c r="U15" t="n">
-        <v>0.033</v>
+        <v>0.035</v>
       </c>
       <c r="V15" t="n">
         <v>0.001</v>
@@ -2215,285 +2119,75 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>U2Net-Saliency</t>
+          <t>grad_cam</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.86</v>
+        <v>0.858</v>
       </c>
       <c r="C16" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.852</v>
       </c>
       <c r="D16" t="n">
-        <v>0.797</v>
+        <v>0.849</v>
       </c>
       <c r="E16" t="n">
-        <v>0.764</v>
+        <v>0.837</v>
       </c>
       <c r="F16" t="n">
-        <v>0.754</v>
+        <v>0.826</v>
       </c>
       <c r="G16" t="n">
-        <v>0.755</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>0.741</v>
+        <v>0.806</v>
       </c>
       <c r="I16" t="n">
-        <v>0.712</v>
+        <v>0.782</v>
       </c>
       <c r="J16" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.772</v>
       </c>
       <c r="K16" t="n">
-        <v>0.666</v>
+        <v>0.752</v>
       </c>
       <c r="L16" t="n">
-        <v>0.608</v>
+        <v>0.729</v>
       </c>
       <c r="M16" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.698</v>
       </c>
       <c r="N16" t="n">
-        <v>0.519</v>
+        <v>0.659</v>
       </c>
       <c r="O16" t="n">
-        <v>0.465</v>
+        <v>0.602</v>
       </c>
       <c r="P16" t="n">
-        <v>0.395</v>
+        <v>0.544</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.31</v>
+        <v>0.464</v>
       </c>
       <c r="R16" t="n">
-        <v>0.237</v>
+        <v>0.382</v>
       </c>
       <c r="S16" t="n">
-        <v>0.151</v>
+        <v>0.248</v>
       </c>
       <c r="T16" t="n">
-        <v>0.081</v>
+        <v>0.127</v>
       </c>
       <c r="U16" t="n">
-        <v>0.036</v>
+        <v>0.032</v>
       </c>
       <c r="V16" t="n">
         <v>0.001</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>inputxgradient_u2net_fill</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0.757</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.716</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.6879999999999999</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0.674</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0.646</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.615</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0.594</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0.5659999999999999</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0.538</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0.527</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.502</v>
-      </c>
-      <c r="N17" t="n">
-        <v>0.456</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0.421</v>
-      </c>
-      <c r="P17" t="n">
-        <v>0.365</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>0.324</v>
-      </c>
-      <c r="R17" t="n">
-        <v>0.246</v>
-      </c>
-      <c r="S17" t="n">
-        <v>0.183</v>
-      </c>
-      <c r="T17" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="U17" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="V17" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>dinov2_COMBO_ENT_SMOOTH</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0.852</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.826</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.805</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0.796</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0.774</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0.756</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0.723</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0.694</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0.663</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0.612</v>
-      </c>
-      <c r="N18" t="n">
-        <v>0.5659999999999999</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0.518</v>
-      </c>
-      <c r="P18" t="n">
-        <v>0.435</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>0.367</v>
-      </c>
-      <c r="R18" t="n">
-        <v>0.295</v>
-      </c>
-      <c r="S18" t="n">
-        <v>0.212</v>
-      </c>
-      <c r="T18" t="n">
-        <v>0.123</v>
-      </c>
-      <c r="U18" t="n">
-        <v>0.051</v>
-      </c>
-      <c r="V18" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>grad_cam</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0.853</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.837</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.828</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0.8149999999999999</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0.8110000000000001</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0.801</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0.783</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0.755</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0.699</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0.663</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="P19" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>0.494</v>
-      </c>
-      <c r="R19" t="n">
-        <v>0.405</v>
-      </c>
-      <c r="S19" t="n">
-        <v>0.276</v>
-      </c>
-      <c r="T19" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="U19" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="V19" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:V19">
+  <conditionalFormatting sqref="B2:V16">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>

</xml_diff>